<commit_message>
feat: variar preguntas de encuesta y actualizar guías de escalas
</commit_message>
<xml_diff>
--- a/ENCUESTA_INSTITUCIONAL_CESU_2025_ACTUALIZADA.xlsx
+++ b/ENCUESTA_INSTITUCIONAL_CESU_2025_ACTUALIZADA.xlsx
@@ -500,7 +500,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica en el proyecto educativo del programa, o lo que haga sus veces, los elementos educativos más relevantes del programa de acuerdo con el ámbito profesional/laboral y/o el académico y el campo de conocimiento y/o en sus entornos sociales y comunitarios..</t>
+          <t>¿Puede identificar en el PEP los elementos formativos clave que responden al campo profesional y al entorno social de su programa? (Escala: Conozco completamente / Conozco bien / Conozco parcialmente / Conozco poco / No conozco)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -515,7 +515,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 1. Proyecto educativo del programa del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su rol dentro de la institución, califique los aspectos relacionados con los recursos informáticos y de comunicación con que cuenta el programa académico, en cuanto a su pertinencia, correspondencia y suficiencia: en coherencia con la actualización del Acuerdo 01 de 2025.</t>
+          <t>¿Qué tan apropiado está el proyecto educativo del programa entre directivos, profesores y estudiantes para orientar decisiones académicas? (Escala: Totalmente apropiado / Apropiado / Parcialmente apropiado / Poco apropiado / Nada apropiado)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Se modifica de '104.  Apreciación de directivos, profesores y estudiantes del programa sobre la pertinencia, correspondencia y suficiencia de los recursos informáticos y de comunicación con que cuenta el programa.' a '2. Evalúa y mejora la apropiación del proyecto educativo del programa, o lo que haga sus veces, por parte de toda la comunidad del programa.' por cambio de alcance/redacción en el Acuerdo 01 de 2025.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra la coherencia con la identidad institucional y las conexiones con las declaraciones del proyecto educativo del programa, o lo que haga sus veces, con el ámbito profesional/laboral y/o el académico y el campo de conocimiento y/o en sus entornos sociales y comunitarios..</t>
+          <t>¿En qué medida las acciones del programa son coherentes con la identidad institucional y con lo declarado en el PEP? (Escala: Totalmente de acuerdo / De acuerdo / Neutral / En desacuerdo / Totalmente en desacuerdo)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 1. Proyecto educativo del programa del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Analiza y sustenta su relevancia y pertinencia a partir de las necesidades locales, regionales, nacionales o internacionales previamente definidas..</t>
+          <t>¿Con qué nivel de sustento el programa demuestra su pertinencia frente a necesidades locales, regionales, nacionales e internacionales? (Escala: Evidencia robusta / Evidencia suficiente / Evidencia parcial / Evidencia limitada / Sin evidencia)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 2. Relevancia académica y pertinencia social del programa académico del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Logra el reconocimiento de actores externos (del ámbito profesional/laboral y/o el académico y el campo de conocimiento y/o en sus entornos sociales y comunitarios)..</t>
+          <t>¿Qué nivel de reconocimiento externo ha alcanzado el programa por su aporte académico y social en los últimos dos años? (Escala: Alto reconocimiento / Reconocimiento moderado / Bajo reconocimiento / Sin reconocimiento / No sé)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 2. Relevancia académica y pertinencia social del programa académico del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica y evalúa los impactos en la formación integral desde la participación de los estudiantes en las distintas actividades que la promueven..</t>
+          <t>En los últimos 6 meses, ¿con qué frecuencia has participado en actividades de formación integral promovidas por el programa? (Escala: Siempre / Frecuentemente / A veces / Rara vez / Nunca)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 3. Incidencia de las actividades de formación integral del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evidencia resultados, logros e impactos en la permanencia y la graduación oportuna en el marco de la normatividad y del contexto del programa, de la caracterización de los estudiantes, y de las estrategias de orientación, acompañamiento y seguimiento acordes con las características particulares de la comunidad de estudiantes..</t>
+          <t>¿Qué tan efectivos han sido el acompañamiento y las estrategias de seguimiento para favorecer tu permanencia y graduación oportuna? (Escala: Muy efectivos / Efectivos / Moderadamente efectivos / Poco efectivos / Nada efectivos)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -737,7 +737,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 4. Orientación, acompañamiento y seguimiento a estudiantes del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su rol dentro de la institución, califique como han sido los medios, espacios y ambientes necesarios para fortalecer en los estudiantes las habilidades y destrezas para el trabajo autónomo.</t>
+          <t>¿Las estrategias pedagógicas del programa fortalecen tu autonomía y trabajo colaborativo en las asignaturas? (Escala: Siempre / Frecuentemente / A veces / Rara vez / Nunca)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Se mantiene del modelo anterior. Coherente con la Característica 5. Estrategias pedagógicas para el fortalecimiento de la autonomía del Acuerdo 01 de 2025.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica y evalúa los resultados, logros e impactos de las políticas académicas y normativas que reconocen y acogen características particulares de la comunidad de estudiantes en el proceso formativo..</t>
+          <t>¿Percibes que las políticas académicas del programa promueven respeto, inclusión y atención a la diversidad durante tu formación? (Escala: Totalmente de acuerdo / De acuerdo / Neutral / En desacuerdo / Totalmente en desacuerdo)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 6. Políticas académicas y normativas en el proceso formativo en procura de una cultura de paz y tolerancia, el antirracismo, la perspectiva de género y la atención a poblaciones diversas, entre otros. El programa académico da cuenta de la divulgación, aplicación y actualización de los reglamentos estudiantiles y las políticas académicas aprobadas, en los que se definen, entre otros aspectos, los deberes y derechos, el régimen disciplinario, la participación de la comunidad académica en la toma de decisiones y las condiciones y exigencias académicas de permanencia, graduación y la generación de una cultura de la paz, la tolerancia, el reconocimiento y el respeto mutuo, el antirracismo, la perspectiva de género e identidades diversas, y la inclusión de personas con discapacidad, entre otros, de acuerdo con las características y modalidad del programa académico del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica los estímulos y apoyos dirigidos a toda la comunidad estudiantil y aquellos con enfoque diferencial..</t>
+          <t>¿Conoces los estímulos y apoyos (académicos, económicos o de bienestar) disponibles para estudiantes del programa? (Escala: Sí, claramente / Sí, parcialmente / Los he escuchado / No los conozco / No sé)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 7. Estímulos y apoyos para todos los estudiantes y en atención a la del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -870,7 +870,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica y evalúa los impactos de los estímulos y apoyos para estudiantes y en atención a la diversidad, el pluralismo y la inclusión de acuerdo con los ajustes razonables..</t>
+          <t>Cuando has requerido apoyo diferencial o ajustes razonables, ¿qué tan pertinente ha sido la respuesta institucional? (Escala: Muy pertinente / Pertinente / Medianamente pertinente / Poco pertinente / Nada pertinente)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 7. Estímulos y apoyos para todos los estudiantes y en atención a la del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evalúa los resultados de los procesos de selección, vinculación y permanencia de los profesores identificando su incidencia en el mejoramiento del programa y en sus procesos y resultados académicos..</t>
+          <t>¿En qué medida los procesos de selección, vinculación y permanencia docente han mejorado los resultados académicos del programa? (Escala: Muy alta / Alta / Media / Baja / Muy baja)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 8. Resultados de los procesos de selección, vinculación y permanencia de los profesores en el mejoramiento del programa del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica la apropiación y conexiones de los docentes con el estatuto, o lo que haga sus veces, y el quehacer profesoral..</t>
+          <t>¿Qué tan bien conoce el estatuto profesoral (o su equivalente) y su relación con las funciones académicas del programa? (Escala: Lo conozco completamente / Lo conozco bien / Lo conozco parcialmente / Lo conozco poco / No lo conozco)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 9. Estatuto, trayectoria y reconocimiento profesoral del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica los efectos de la aplicación del estatuto profesoral, o lo que haga sus veces, en la trayectoria profesoral, la inclusión, el reconocimiento de los méritos y el ascenso en el escalafón y los que se declaren en las normativas relacionadas..</t>
+          <t>¿La aplicación del estatuto profesoral ha favorecido una trayectoria docente con reconocimiento de méritos y oportunidades de ascenso? (Escala: Totalmente de acuerdo / De acuerdo / Neutral / En desacuerdo / Totalmente en desacuerdo)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 9. Estatuto, trayectoria y reconocimiento profesoral del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra que cuenta con una planta profesoral que, en número, tipo de vinculación, formación y contratación es coherente con las características propias del programa, su campo de formación, las labores misionales y la totalidad de los estudiantes matriculados..</t>
+          <t>¿La planta profesoral actual es suficiente y pertinente para atender la totalidad de estudiantes y labores misionales del programa? (Escala: Totalmente suficiente / Suficiente / Parcialmente suficiente / Insuficiente / Críticamente insuficiente)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 10. Planta profesoral para materializar el proyecto educativo del del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra resultados, logros e impactos de actividades realizadas en el programa por profesores que contribuyen a la materialización del proyecto educativo del programa, o lo que haga sus veces..</t>
+          <t>¿Qué impacto han tenido las actividades desarrolladas por los profesores en la materialización del proyecto educativo del programa? (Escala: Alto impacto / Impacto moderado / Bajo impacto / Sin impacto observable / No aplica)</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 10. Planta profesoral para materializar el proyecto educativo del del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica los programas y acciones relacionadas con el desarrollo profesoral en coherencia con las políticas institucionales..</t>
+          <t>¿Con qué frecuencia participa en programas institucionales de desarrollo profesoral alineados con las políticas vigentes? (Escala: Siempre / Frecuentemente / A veces / Rara vez / Nunca)</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 11. Capacidades, procesos, y resultados, del desarrollo profesoral del del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica y evalúa los resultados en la implementación de las políticas relacionadas con el desarrollo profesoral y su contribución al mejoramiento del programa..</t>
+          <t>¿Qué tan efectivos han sido los programas de desarrollo profesoral para mejorar la calidad del programa? (Escala: Muy efectivos / Efectivos / Moderadamente efectivos / Poco efectivos / Nada efectivos)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 11. Capacidades, procesos, y resultados, del desarrollo profesoral del del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1166,7 +1166,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra la coherencia entre los estímulos a la trayectoria de los profesores con los procesos y resultados académicos y evidencia su contribución al mejoramiento del programa..</t>
+          <t>¿Los estímulos a la trayectoria docente están alineados con los resultados académicos que el programa busca fortalecer? (Escala: Totalmente alineados / Alineados / Parcialmente alineados / Poco alineados / Nada alineados)</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 12. Coherencia entre los estímulos a la trayectoria de los profesores del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Fomenta, apoya y evalúa la producción del material docente de acuerdo con las características y modalidad del programa académico..</t>
+          <t>¿Qué tan adecuado es el apoyo institucional para producir material docente individual y colaborativo en el programa? (Escala: Muy adecuado / Adecuado / Medianamente adecuado / Poco adecuado / Nada adecuado)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 13. Producción, pertinencia, utilización e impacto de material docente. Los profesores producen de manera individual y colaborativa con otros del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica y evalúa los impactos del material docente en los procesos y resultados académicos..</t>
+          <t>¿El material docente producido por los profesores mejora de forma verificable los procesos y resultados académicos? (Escala: Siempre / Frecuentemente / A veces / Rara vez / Nunca)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 13. Producción, pertinencia, utilización e impacto de material docente. Los profesores producen de manera individual y colaborativa con otros del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra como la evaluación integral docente mejora el desempeño de la planta docente y sus efectos sobre la calidad del programa..</t>
+          <t>¿En qué medida la evaluación integral docente ha contribuido a mejorar el desempeño de la planta profesoral? (Escala: Contribución muy alta / Alta / Media / Baja / Nula)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 14. Evaluación integral de profesores y sus efectos en el mejoramiento del programa del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evalúa de manera integral a los profesores en las distintas labores e identifica los efectos sobre la calidad del programa y la mejora en las prácticas pedagógicas, la permanencia, en la trayectoria, entre otros..</t>
+          <t>¿Los resultados de la evaluación docente se traducen en cambios concretos en prácticas pedagógicas y calidad del programa? (Escala: Siempre / Frecuentemente / A veces / Rara vez / Nunca)</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 14. Evaluación integral de profesores y sus efectos en el mejoramiento del programa del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra un seguimiento permanente y representativo a la ubicación, realizaciones, redes, logros e impactos de sus egresados y sus contribuciones al mejoramiento del programa..</t>
+          <t>¿Con qué periodicidad el programa realiza seguimiento a su trayectoria laboral y aportes como egresado? (Escala: Semestral / Anual / Esporádico / Casi nunca / Nunca)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 15. Seguimiento de los egresados, su caracterización y aportes en el del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evidencia el reconocimiento al desempeño y evalúa el aporte de los egresados a la solución de los problemas económicos, ambientales, tecnológicos, sociales y culturales, a través del ejercicio de la disciplina, profesión, ocupación u oficio correspondiente..</t>
+          <t>Desde su experiencia, ¿qué tan reconocido es el desempeño de los egresados del programa en la solución de problemáticas del entorno? (Escala: Muy reconocido / Reconocido / Medianamente reconocido / Poco reconocido / No reconocido)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 16. Impacto y reconocimientos obtenidos por los egresados en el del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra los efectos de la evaluación de la gestión curricular en la mejora del programa..</t>
+          <t>¿La evaluación de la gestión curricular ha generado mejoras reales en integralidad, flexibilidad e interacción disciplinar del programa? (Escala: Totalmente de acuerdo / De acuerdo / Neutral / En desacuerdo / Totalmente en desacuerdo)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 17. Evaluación de la gestión curricular y sus efectos en la mejora del programa desde una perspectiva de integralidad, flexibilidad e interacción de las del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1462,7 +1462,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evalúa la pertinencia de la definición de la denominación, la duración y el número de créditos desde una perspectiva de integralidad, flexibilidad e interacción de las disciplinas..</t>
+          <t>¿Qué tan pertinente considera la denominación, duración y número de créditos del programa frente a su propósito formativo? (Escala: Muy pertinente / Pertinente / Moderadamente pertinente / Poco pertinente / Nada pertinente)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 17. Evaluación de la gestión curricular y sus efectos en la mejora del programa desde una perspectiva de integralidad, flexibilidad e interacción de las del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evalúa los efectos de las modificaciones realizadas en los aspectos académicos y de evaluación del programa..</t>
+          <t>¿Las modificaciones recientes en aspectos académicos y de evaluación han mejorado el aprendizaje de manera observable? (Escala: Mejoró mucho / Mejoró / Mejoró poco / No mejoró / Empeoró)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 17. Evaluación de la gestión curricular y sus efectos en la mejora del programa desde una perspectiva de integralidad, flexibilidad e interacción de las del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1536,7 +1536,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra que las estrategias pedagógicas responden a las características particulares de la oferta del programa, la formación de los profesores de la comunidad de estudiantes e incorpora los resultados de las investigaciones pedagógicas institucionales en conexión con el proyecto educativo institucional y el proyecto educativo del programa, o lo que haga sus veces..</t>
+          <t>¿Las estrategias pedagógicas del programa responden al perfil de estudiantes y se articulan con el proyecto educativo institucional y del programa? (Escala: Siempre / Frecuentemente / A veces / Rara vez / Nunca)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 18. Coherencia de las estrategias pedagógicas con el proyecto educativo del programa académico y las características de la comunidad de estudiantes del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evidencia sistemas de evaluación que integren procedimientos claros y transparentes, dan cuenta de los procesos y resultados académicos con innovaciones que generan transformaciones profundas en el aprendizaje, facilitar la inclusión y acoger las dinámicas y cambios particulares de los campos del conocimiento..</t>
+          <t>¿El sistema de evaluación estudiantil es claro, transparente e innovador para valorar conocimientos, capacidades y habilidades? (Escala: Totalmente de acuerdo / De acuerdo / Neutral / En desacuerdo / Totalmente en desacuerdo)</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 19. Sistema de evaluación de estudiantes en coherencia con las transformaciones en las teorías y métodos de aprendizaje, las dinámicas del contexto y las declaraciones del programa. El programa académico cuenta con un sistema de evaluación de estudiantes basado en políticas y normas claras, universales y transparentes. Dicho sistema permite valorar periódica o permanentemente los procesos y resultados académicos, las actitudes, los conocimientos, las capacidades y las habilidades adquiridas por los estudiantes en coherencia con los objetivos de formación previstos. Los sistemas de evaluación integran la innovación para generar del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra los efectos de la evaluación sistemática y permanente de los procesos y resultados académicos en la mejora del programa.</t>
+          <t>¿Qué efecto tiene la evaluación sistemática de procesos y resultados académicos sobre el mejoramiento continuo del programa? (Escala: Muy alto / Alto / Medio / Bajo / Nulo)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 20. Aportes del sistema de evaluación de los procesos y resultados del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra los efectos del diseño curricular en el cumplimiento de los propósitos del proyecto educativo del programa, o lo que haga sus veces, y el perfil de egreso, y los evidencia a través de los estudios de desempeño de los egresados..</t>
+          <t>¿El diseño curricular permite cumplir el perfil de egreso y las competencias previstas en el proyecto educativo del programa? (Escala: Totalmente / En gran medida / Parcialmente / En baja medida / No permite)</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 21. Coherencia entre las competencias, capacidades, habilidades y/o destrezas, los procesos y resultados académicos previstos y demás aspectos curriculares definidos en el proyecto educativo del programa académico del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1684,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica los resultados y logros y evalúa los impactos de las políticas y estrategias implementadas para la permanencia y la graduación de los estudiantes atendiendo criterios de equidad e inclusión..</t>
+          <t>¿Ha recibido apoyos institucionales con enfoque de equidad e inclusión que hayan favorecido su permanencia y graduación? (Escala: Sí, múltiples apoyos / Sí, un apoyo clave / Sí, apoyo limitado / No he recibido / No sé)</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 22. Impacto de las políticas y estrategias implementadas para la permanencia y la graduación. El programa académico demuestra la existencia, los resultados y las evidencias de impacto de las políticas de bienestar, permanencia y graduación, de los programas de apoyo que pueden tener, por ejemplo, enfoques diferenciales, accesibles, interculturales, plurilingües, territoriales e interseccionales para la permanencia con equidad fundada en una educación inclusiva, y la graduación de los estudiantes, que incorporan, entre otros, procesos de inducción, acompañamiento, orientación vocacional, adaptación a la vida universitaria, orientación para el trabajo de grado y práctica laboral del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra la existencia de un sistema de alertas tempranas para la prevención y atención diferenciada de los estudiantes y da cuenta de su efectividad..</t>
+          <t>¿El sistema de alertas tempranas identifica y atiende oportunamente a estudiantes en riesgo de deserción? (Escala: Muy efectivo / Efectivo / Moderadamente efectivo / Poco efectivo / Nada efectivo)</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 23. Caracterización y atención de estudiantes a través de los sistemas, estrategias y programas dispuestos para tal fin del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra el impacto de la caracterización a lo largo del proceso formativo de los estudiantes en la determinación de las estrategias y apoyos que promueven la permanencia y graduación oportuna..</t>
+          <t>¿La caracterización de estudiantes se usa realmente para definir apoyos y estrategias de permanencia durante su proceso formativo? (Escala: Siempre / Frecuentemente / A veces / Rara vez / Nunca)</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1773,7 +1773,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 23. Caracterización y atención de estudiantes a través de los sistemas, estrategias y programas dispuestos para tal fin del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1795,7 +1795,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra el impacto de los programas de permanencia y graduación en la evolución de las transformaciones curriculares y pedagógicas, en el marco de una formación integral..</t>
+          <t>¿Los programas de permanencia y graduación han impulsado ajustes curriculares y pedagógicos útiles para su formación integral? (Escala: Totalmente de acuerdo / De acuerdo / Neutral / En desacuerdo / Totalmente en desacuerdo)</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 24. Evolución de los ajustes a los aspectos curriculares y pedagógicos como resultado de los programas de permanencia y graduación del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra la contribución efectiva de los mecanismos de selección con criterios de equidad e inclusión en el desarrollo de actividades orientadas a la reducción de la deserción y a la graduación oportuna..</t>
+          <t>¿Los mecanismos de selección del programa contribuyen a reducir la deserción y promover la graduación oportuna con criterios de inclusión? (Escala: Contribuyen mucho / Contribuyen / Contribuyen poco / No contribuyen / No sé)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 25. Contribución de los mecanismos de selección a la reducción de del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1869,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evidencia la Incorporación de las tendencias de contextos locales, regionales, nacionales e internacionales en la actualización de los aspectos curriculares, a partir de espacios de reflexión y análisis..</t>
+          <t>¿Qué tan incorporadas están las tendencias académicas y profesionales del contexto local, nacional e internacional en la actualización curricular del programa? (Escala: Muy incorporadas / Incorporadas / Parcialmente incorporadas / Poco incorporadas / No incorporadas)</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 26. Inserción del programa en contextos académicos locales, regionales, nacionales e internacionales. El programa académico da cuenta de que en la reflexión, organización y actualización de sus aspectos curriculares toma como referencia las tendencias, el estado del arte de la disciplina o profesión y los indicadores de calidad reconocidos por la comunidad académica nacional e internacional del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1906,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evidencia y evalúa el impacto en la cooperación de profesores y estudiantes con otras instituciones o entidades locales, regionales, nacionales y extranjeras en el desarrollo de las labores del programa..</t>
+          <t>¿Qué impacto han tenido las alianzas y cooperaciones de profesores y estudiantes con otras instituciones en el posicionamiento del programa? (Escala: Alto impacto / Impacto moderado / Bajo impacto / Sin impacto observable / No sé)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 27. Resultados y logros de las relaciones y de la cooperación de profesores y estudiantes con comunidades locales, regionales, nacionales y extranjeras y sus efectos en el posicionamiento del programa del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica y evalúa los impactos de las políticas institucionales el desarrollo de habilidades comunicativas en una o varias lenguas en coherencia con sus declaraciones.</t>
+          <t>¿Las políticas institucionales para fortalecer habilidades comunicativas en una o varias lenguas muestran resultados verificables en el programa? (Escala: Siempre / Frecuentemente / A veces / Rara vez / Nunca)</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 28. Efectos de las políticas para el desarrollo de habilidades comunicativas en una o varias lenguas en coherencia con el proyecto educativo del programa académico del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su rol dentro de la institución, califique el nivel de impacto que tienen las prácticas pedagógicas en el fortalecimiento de las competencias en los estudiantes, y, el aporte de estas a las comunidades donde las realizan en coherencia con la actualización del Acuerdo 01 de 2025.</t>
+          <t>¿En qué medida los proyectos de extensión e interacción social del programa aportan a la solución de problemas del entorno? (Escala: En muy alta medida / En alta medida / En medida media / En baja medida / En ninguna medida)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Se modifica de '49. Evidencia de la evaluación y el mejoramiento de las estrategias y prácticas pedagógicas, a partir de los aportes de la investigación pedagógica y de los procesos de actualización de los profesores.' a '41. Identifica y evalúa los impactos y los aportes de la extensión y la proyección e interacción social en la solución de los problemas y la transformación de sus contextos.' por cambio de alcance/redacción en el Acuerdo 01 de 2025.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica y evalúa los impactos que tiene la participación de los estudiantes en las actividades de extensión, proyección e interacción social sobre sus procesos de formación..</t>
+          <t>Desde su observación externa, ¿la participación estudiantil en actividades de extensión mejora las competencias profesionales de los futuros egresados? (Escala: Sí, claramente / Sí, parcialmente / Se observa poco / No se observa / No sabe)</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 29. Impacto y aportes de la proyección e interacción social en del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evalúa la consolidación y la evolución de las condiciones y los recursos para el desarrollo de actividades de investigación, la innovación, el desarrollo tecnológico, la creación e investigación-creación artística y cultural, de los profesores del programa, reconocidas por el Sistema Nacional de Ciencia, Tecnología e Innovación..</t>
+          <t>¿Las condiciones y recursos para investigación, innovación y creación de los profesores son suficientes y sostenidos en el tiempo? (Escala: Totalmente suficientes / Suficientes / Parcialmente suficientes / Insuficientes / Muy insuficientes)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 30. Capacidades y procesos para la consolidación de la investigación, el desarrollo tecnológico, la innovación, la creación e investigación creación artística y cultural en el programa académico. El programa académico demuestra que los profesores realizan actividades de investigación, desarrollo tecnológico, innovación o creación, reconocidas por el Sistema Nacional de Ciencia y Tecnología, y cuenta con condiciones y recursos institucionales para el desarrollo de dichas actividades del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evidencia los resultados, logros e impactos de la investigación, el desarrollo tecnológico, la innovación, la creación e investigación creación artística y cultural que contribuyen a la actualización y generación de conocimiento o a la solución de problemas de la sociedad, la generación de nuevos espacios para la renovación permanente de enfoques conceptuales y teóricos que contribuyan al desarrollo investigativo innovador y a la producción intelectual..</t>
+          <t>¿Qué tan visibles son los resultados de investigación e innovación del programa en la actualización del conocimiento y la solución de problemas sociales? (Escala: Muy visibles / Visibles / Medianamente visibles / Poco visibles / No visibles)</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 31. Identificación de los resultados, logros e impactos de la investigación, el desarrollo tecnológico, la innovación, la creación e investigación creación artística y cultural en los diferentes contextos del programa. El programa académico evidencia que los productos resultantes de la investigación, el desarrollo tecnológico, la innovación y la creación enriquecen los aspectos curriculares, fortalecen la formación de los estudiantes y contribuyen a la actualización y generación de conocimiento o a la solución de problemas de la sociedad, la generación de nuevos espacios para la renovación permanente de enfoques conceptuales y teóricos que contribuyan al desarrollo investigativo innovador y a la producción intelectual del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evalúa los resultados, logros e impactos de la investigación, el desarrollo tecnológico, la innovación, la creación e investigación creación artística y cultural sobre la formación de los estudiantes..</t>
+          <t>¿La investigación y creación desarrollada por el programa fortalece de forma efectiva la formación de sus estudiantes? (Escala: Muy efectiva / Efectiva / Moderadamente efectiva / Poco efectiva / Nada efectiva)</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 31. Identificación de los resultados, logros e impactos de la investigación, el desarrollo tecnológico, la innovación, la creación e investigación creación artística y cultural en los diferentes contextos del programa. El programa académico evidencia que los productos resultantes de la investigación, el desarrollo tecnológico, la innovación y la creación enriquecen los aspectos curriculares, fortalecen la formación de los estudiantes y contribuyen a la actualización y generación de conocimiento o a la solución de problemas de la sociedad, la generación de nuevos espacios para la renovación permanente de enfoques conceptuales y teóricos que contribuyan al desarrollo investigativo innovador y a la producción intelectual del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2165,7 +2165,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Articula los propósitos académicos con las dinámicas investigativas desde los productos y actividades asociados a las líneas de investigación con las declaraciones del programa..</t>
+          <t>¿Las líneas de investigación del programa se articulan con los propósitos académicos y con lo declarado en el proyecto educativo? (Escala: Totalmente articuladas / Articuladas / Parcialmente articuladas / Poco articuladas / No articuladas)</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 32. Coherencia de las líneas de investigación y/o creación y del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2202,7 +2202,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Consolida la participación de la comunidad de estudiantes en las actividades de formación para la investigación, la innovación, el desarrollo tecnológico, la creación e investigación-creación artística y cultural..</t>
+          <t>¿Con qué frecuencia los estudiantes participan en semilleros, proyectos o actividades de formación para la investigación e innovación? (Escala: Siempre / Frecuentemente / A veces / Rara vez / Nunca)</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 33. Resultados de la formación para la investigación, desarrollo tecnológico, la innovación y la creación del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2239,7 +2239,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica y sistematiza los resultados de la formación para la investigación, la innovación, el desarrollo tecnológico, la creación e investigación-creación artística y cultural de los estudiantes del programa..</t>
+          <t>¿El programa sistematiza y usa resultados de formación investigativa estudiantil para tomar decisiones académicas? (Escala: Siempre / Frecuentemente / A veces / Rara vez / Nunca)</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 33. Resultados de la formación para la investigación, desarrollo tecnológico, la innovación y la creación del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Incorpora e implementa los resultados de investigación, el desarrollo tecnológico, la innovación y/o la creación e investigación-creación artística y cultural en el mejoramiento del programa..</t>
+          <t>¿Con qué nivel de efectividad se aplican resultados de investigación e innovación para mejorar contenidos, metodologías o procesos del programa? (Escala: Muy alta / Alta / Media / Baja / Nula)</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 34. Demostración del uso de los resultados de investigación, el desarrollo tecnológico, la innovación y/o la creación e investigación-creación artística y cultural en el mejoramiento del programa del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2313,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evalúa la pertinencia y el impacto de los resultados investigación, el desarrollo tecnológico, la innovación y/o la creación e investigación-creación artística y cultural en los contextos del programa..</t>
+          <t>¿Qué impacto evidencian los proyectos de investigación y creación del programa en su contexto territorial y sectorial? (Escala: Alto impacto / Impacto moderado / Bajo impacto / Sin impacto observable / No se dispone de evidencia)</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 35. Impacto de la investigación y/o la investigación-creación en el contexto en el que se ofrece el programa. El programa académico da cuenta de los impactos generados en su contexto o entorno, de los resultados alcanzados en el periodo de observación, de los desarrollos de los proyectos de investigación asociados coherentemente a las líneas de investigación manifiestos en su proyecto educativo, o en lo que haga sus veces del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2350,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evalúa la implementación de las políticas relacionadas con los programas y servicios de bienestar en el marco del pluralismo, la diversidad y la inclusión, basado en el nivel de participación de la comunidad del programa..</t>
+          <t>¿Qué tan satisfactoria ha sido la implementación de programas y servicios de bienestar con enfoque de diversidad e inclusión en el programa? (Escala: Muy satisfactoria / Satisfactoria / Neutra / Insatisfactoria / Muy insatisfactoria)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 36. Evolución y evaluación de los programas y servicios que desarrollan las políticas de bienestar en el marco del pluralismo, la diversidad y la del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evalúa la evolución de los programas y servicios de bienestar en el marco del pluralismo, la diversidad y la inclusión, basado en el nivel de participación de la comunidad del programa..</t>
+          <t>En comparación con periodos anteriores, ¿cómo valora la evolución de los programas y servicios de bienestar dirigidos a la comunidad del programa? (Escala: Mejoró significativamente / Mejoró / Se mantiene / Empeoró / Empeoró significativamente)</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 36. Evolución y evaluación de los programas y servicios que desarrollan las políticas de bienestar en el marco del pluralismo, la diversidad y la del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2424,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica y evalúa los impactos de los programas, planes y actividades de bienestar en la formación integral y en la calidad de vida de la comunidad de estudiantes..</t>
+          <t>¿Los programas de bienestar han mejorado su formación integral y calidad de vida como estudiante? (Escala: Mucho / Bastante / Algo / Poco / Nada)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 37. Incidencia de los programas, planes y actividades de bienestar en la formación integral y en la calidad de vida de la comunidad de estudiantes. El del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Consolida y demuestra el avance de la infraestructura, los programas y servicios con los que desarrollan las políticas de bienestar en el marco del pluralismo, la diversidad y la inclusión, teniendo como referencia las características particulares de toda la comunidad del programa y las que determinan su oferta..</t>
+          <t>¿Las actividades, servicios e infraestructura de bienestar están adaptados a las características y necesidades de la comunidad del programa? (Escala: Totalmente adaptados / Adaptados / Parcialmente adaptados / Poco adaptados / No adaptados)</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 38. Adaptación y evaluación de los programas, actividades e infraestructura de bienestar a las condiciones particulares que determinan la del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2498,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evalúa la pertinencia y la actualización de los medios educativos que soportan.</t>
+          <t>¿Los medios educativos del programa se mantienen actualizados y pertinentes para el aprendizaje en su modalidad de formación? (Escala: Siempre / Frecuentemente / A veces / Rara vez / Nunca)</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -2513,7 +2513,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 39. Evolución y evaluación de los medios educativos que soportan del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2535,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica y evalúa los efectos de los medios educativos en los procesos y resultados académicos de los estudiantes atendiendo su contexto..</t>
+          <t>¿Qué tan efectivos son los medios educativos para mejorar sus procesos y resultados académicos en su contexto? (Escala: Muy efectivos / Efectivos / Moderadamente efectivos / Poco efectivos / Nada efectivos)</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 40. Aporte de los medios educativos en los procesos y resultados académicos de los estudiantes atendiendo su contexto y a los principios rectores del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2572,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evalúa de la idoneidad, el uso, la usabilidad, la suficiencia y la calidad de los medios educativos, recursos bibliográficos y de información y de los servicios asociados, en coherencia con las características particulares de la comunidad del programa, y las que determinan su oferta..</t>
+          <t>¿Cómo evalúa la idoneidad, usabilidad y suficiencia de recursos bibliográficos, de información y servicios asociados del programa? (Escala: Excelente / Buena / Aceptable / Deficiente / Muy deficiente)</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 41. Evolución de la suficiencia y calidad de los medios educativos, recursos bibliográficos y de información en coherencia con las dinámicas propias del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evalúa de la pertinencia, el uso, la usabilidad, la suficiencia, la actualización, el.</t>
+          <t>¿La infraestructura física y tecnológica disponible responde al uso real del programa y a las necesidades de aprendizaje de los estudiantes? (Escala: Totalmente / En gran medida / Parcialmente / En baja medida / No responde)</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 42. Evolución, suficiencia y evaluación de los recursos de infraestructura física y tecnológica en coherencia con el proyecto educativo del del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica y evalúa los principales logros y resultados de la organización y la gestión del programa..</t>
+          <t>¿Con qué nivel de cumplimiento la organización del programa alcanza sus metas de gestión académica y administrativa? (Escala: Muy alto / Alto / Medio / Bajo / Muy bajo)</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 43. Identificación de los logros y resultados de la organización y la gestión del programa. El programa académico cuenta con una estructura organizacional con cuerpo(s) colegiado(s) donde participan por lo menos representantes de los profesores, los estudiantes y los egresados, y que, además, tiene implementados los mecanismos administrativos necesarios para identificar los logros y resultados de la organización y la gestión del programa del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2683,7 +2683,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Evidencia la participación en los cuerpos (s) colegiado(s) de los representantes de los profesores, los estudiantes y los egresados y su contribución a los planes de mejoramiento del programa..</t>
+          <t>¿La participación de profesores, estudiantes y egresados en cuerpos colegiados influye en decisiones y planes de mejoramiento del programa? (Escala: Influye mucho / Influye / Influye poco / No influye / No sabe)</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 43. Identificación de los logros y resultados de la organización y la gestión del programa. El programa académico cuenta con una estructura organizacional con cuerpo(s) colegiado(s) donde participan por lo menos representantes de los profesores, los estudiantes y los egresados, y que, además, tiene implementados los mecanismos administrativos necesarios para identificar los logros y resultados de la organización y la gestión del programa del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2720,7 +2720,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Consolida y demuestra el avance de la sostenibilidad, los recursos y las capacidades en coherencia con las características particulares de la comunidad del programa, las que determinan su oferta y su crecimiento o los desafíos del contexto..</t>
+          <t>¿Las capacidades humanas, tecnológicas y de infraestructura del programa muestran sostenibilidad para atender su crecimiento y retos del contexto? (Escala: Totalmente sostenibles / Sostenibles / Parcialmente sostenibles / Poco sostenibles / No sostenibles)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 44. Evolución y evaluación de la sostenibilidad, los recursos y las capacidades del programa en coherencia con el proyecto educativo. El programa académico muestra la evolución y evaluación de la sostenibilidad de las capacidades institucionales en materia de sus recursos humanos, técnicos, tecnológicos, biográficos y de laboratorios, así como de la infraestructura física, entre otros, necesarios para favorecer la permanencia, el desarrollo académico y la graduación de los estudiantes del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Indique su nivel de satisfacción acerca de la suficiencia y calidad de los recursos y sistemas de comunicación e información en la Institución en coherencia con la actualización del Acuerdo 01 de 2025.</t>
+          <t>¿Qué tan efectivo es el liderazgo directivo para consolidar comunidad académica, cultura de calidad y mejoramiento continuo? (Escala: Muy efectivo / Efectivo / Moderadamente efectivo / Poco efectivo / Nada efectivo)</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Se modifica de '92.  Presentación de estudios de satisfacción de profesores y estudiantes del programa acerca de la suficiencia y calidad de los recursos y sistemas de comunicación e información.' a '62. Evalúa el impacto del liderazgo en la dirección y gestión en la consolidación de la comunidad académica del programa y en cultura de la calidad y en los procesos de mejoramiento.' por cambio de alcance/redacción en el Acuerdo 01 de 2025.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra la accesibilidad, consistencia, actualización y protección de los datos en sistemas de información y sus contribuciones a la toma de decisiones para la autorregulación, autoevaluación y el mejoramiento permanente..</t>
+          <t>¿El sistema de información institucional ofrece datos confiables, actualizados, protegidos y oportunos para la toma de decisiones del programa? (Escala: Siempre / Frecuentemente / A veces / Rara vez / Nunca)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 46. Sistemas de comunicación e información actualizados, accesibles y oportunos en el mejoramiento del programa del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2831,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra la efectividad de los sistemas de comunicación en coherencia con las características particulares de la comunidad del programa, las que determinan su oferta..</t>
+          <t>¿Los canales de comunicación del programa son oportunos, accesibles y útiles para la gestión académica y administrativa? (Escala: Totalmente de acuerdo / De acuerdo / Neutral / En desacuerdo / Totalmente en desacuerdo)</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 46. Sistemas de comunicación e información actualizados, accesibles y oportunos en el mejoramiento del programa del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica el impacto de los recursos en la permanencia, el desarrollo académico y la graduación oportuna de los estudiantes, en coherencia con la evolución del programa..</t>
+          <t>¿En qué medida los recursos y capacidades del programa apoyan la permanencia, el desarrollo académico y la graduación oportuna? (Escala: En muy alta medida / En alta medida / En medida media / En baja medida / En ninguna medida)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 47. Consolidación de los recursos y capacidades coherentes con la del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2905,7 +2905,7 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra que dispone de los recursos financieros de funcionamiento e inversión, necesarios para el desarrollo del programa y desarrolla procesos de planeación, seguimiento y ejecución de dichos recursos en coherencia con las dinámicas propias del programa y sus planes de mejoramiento..</t>
+          <t>¿El programa cuenta con sostenibilidad financiera y seguimiento presupuestal suficiente para cumplir sus planes de desarrollo y mejoramiento? (Escala: Sí, plenamente / Sí, con limitaciones menores / Parcialmente / No suficientemente / No)</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 48. Identificación de la sostenibilidad financiera del programa del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2942,7 +2942,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Presenta y evalúa resultados de la participación representativa, reflexiva y critica de la comunidad académica del programa en los procesos de autorregulación, autoevaluación y mejoramiento permanente, para promover una cultura de la calidad y contribuir a la consolidación del sistema interno de aseguramiento de la calidad..</t>
+          <t>¿Qué tan representativa y crítica es la participación de la comunidad académica en autoevaluación, autorregulación y mejoramiento permanente del programa? (Escala: Muy alta / Alta / Media / Baja / Nula)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 49. Reflexión y participación de la comunidad en los procesos de gestión, autoevaluación, autorregulación y mejoramiento permanente del del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Demuestra la evolución y la consolidación de la información y los datos en el marco del sistema interno de aseguramiento de la calidad, para soportar los procesos de autoevaluación, autorregulación y del mejoramiento permanente del programa académico..</t>
+          <t>¿La información consolidada en el sistema interno de aseguramiento de la calidad permite sustentar decisiones de autoevaluación y autorregulación del programa? (Escala: Totalmente / En gran medida / Parcialmente / En baja medida / No permite)</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 50. Consolidación de la información y los datos que dan cuenta de los resultados, logros e impactos de la alta calidad del programa en el periodo de observación correspondiente a la autoevaluación. El programa académico demuestra que ha consolidado la información y los datos en el marco del Sistema Interno de Aseguramiento de la Calidad Institucional para soportar los procesos de autoevaluación, autorregulación y del mejoramiento permanente del programa académico del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Identifica los principales resultados y logros y evalúa los impactos de la cultura de la calidad en el mejoramiento del programa..</t>
+          <t>¿Qué resultados concretos evidencia el programa sobre la cultura de la calidad en sus procesos de mejoramiento? (Escala: Resultados sobresalientes / Resultados sólidos / Resultados parciales / Resultados incipientes / Sin resultados)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 51. Identificación de los principales resultados, logros e impactos de la cultura de la calidad en el mejoramiento del programa. El programa académico del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>
@@ -3053,7 +3053,7 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>De acuerdo con su experiencia, califique en qué medida el programa evidencia el siguiente aspecto: Implementa las recomendaciones realizadas en los procesos de autoevaluación, y realiza un seguimiento que permite evaluar sus efectos sobre mejoramiento permanente del programa..</t>
+          <t>¿Se implementan y monitorean las recomendaciones de autoevaluación hasta verificar su efecto en el mejoramiento permanente del programa? (Escala: Siempre / Frecuentemente / A veces / Rara vez / Nunca)</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Se añade según la Característica 51. Identificación de los principales resultados, logros e impactos de la cultura de la calidad en el mejoramiento del programa. El programa académico del Acuerdo 01 de 2025. No existía en el modelo anterior un aspecto equivalente con trazabilidad directa.</t>
+          <t>Se reformuló para mayor especificidad y variación en la formulación, evitando repetición genérica y adaptándola al actor específico.</t>
         </is>
       </c>
     </row>

</xml_diff>